<commit_message>
Global Search import: pure 1:1 format match to FD/SF (drop ID columns)
Make testrail-import/global-search-v2-testrail-import.csv/.xlsx a pure 1:1
format match to the fees-discounts and simple-flow imports: the 8 named
columns (Title, Section, Type, Priority, Preconditions, Steps, Expected
Result, References) + 2 trailing blank/unnamed columns. Drops the 3
Global-Search-specific ID columns (Internal ID / TestRail Case ID /
TestRail Link); traceability now relies solely on
build/global-search/testrail-id-map.csv per Standing Rule 8, same as the
other two projects. Header byte-identical to FD/SF; 86 data rows; API
cases under the em-dash 'API — Global Search Endpoint' section;
VIU-word-free + feature-flag-free; CRLF row terminators + LF in cells;
deterministic re-run. Docs (PROJECT-STATE.md, CLAUDE.md) updated to
reflect the pure-1:1 format.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/global-search-v2-testrail-import.xlsx
+++ b/testrail-import/global-search-v2-testrail-import.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K87"/>
+  <dimension ref="A1:J87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -439,9 +439,8 @@
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -485,21 +484,8 @@
           <t>References</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Internal ID</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>TestRail Case ID</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>TestRail Link</t>
-        </is>
-      </c>
+      <c r="I1" s="1" t="inlineStr"/>
+      <c r="J1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -549,17 +535,8 @@
           <t>requirements.md 5.1 Trigger and Surface; 8 Functional Requirements</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>GS-KEY-01</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -607,17 +584,8 @@
           <t>requirements.md 5.1 Trigger and Surface</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>GS-KEY-02</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -663,17 +631,8 @@
           <t>requirements.md 5.1; 5.5 Keyboard Navigation</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>GS-KEY-03</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -718,17 +677,8 @@
           <t>requirements.md 5.1 (Esc, clicking underlay, or Cmd+K again closes it)</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>GS-KEY-04</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -774,17 +724,8 @@
           <t>requirements.md 5.1 (clicking the page underlay closes it)</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>GS-KEY-05</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -833,17 +774,8 @@
           <t>requirements.md 5.5 (Up/Down moves focus through visible rows, skipping group headers)</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>GS-KEY-06</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -889,17 +821,8 @@
           <t>requirements.md 5.5 (Enter opens the focused row in the same tab)</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>GS-KEY-07</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -945,17 +868,8 @@
           <t>requirements.md 5.5 (Cmd+Enter or Ctrl+Enter opens in a new browser tab)</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>GS-KEY-08</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1005,17 +919,8 @@
           <t>requirements.md 5.5 (Tab moves focus to the scope tab strip; Left/Right cycles tabs when focus is on the tab strip)</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>GS-KEY-09</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1061,17 +966,8 @@
           <t>requirements.md 5.1 (footer always shows the keyboard legend)</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>GS-KEY-10</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1115,17 +1011,8 @@
           <t>requirements.md 5.2 State 3 (tab strip); design-notes cross-reference</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>GS-TAB-01</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1172,17 +1059,8 @@
           <t>requirements.md 5.2 State 3; 6.2 group order</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>GS-TAB-02</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1227,17 +1105,8 @@
           <t>requirements.md 5.2 State 3 (selecting a tab scopes the query to that entity type)</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>GS-TAB-03</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1282,17 +1151,8 @@
           <t>requirements.md 5.2 State 3</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>GS-TAB-04</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1337,17 +1197,8 @@
           <t>requirements.md 5.2 State 3</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>GS-TAB-05</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1392,17 +1243,8 @@
           <t>requirements.md 5.2 State 3</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>GS-TAB-06</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1447,17 +1289,8 @@
           <t>requirements.md 5.2 State 3</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>GS-TAB-07</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1503,17 +1336,8 @@
           <t>requirements.md 4 (Part Sales is a NEW searchable entity); 5.2 State 3</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>GS-TAB-08</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1559,17 +1383,8 @@
           <t>requirements.md 5.2 State 3 (results grouped by entity type with a count)</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>GS-GRP-01</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1615,17 +1430,8 @@
           <t>requirements.md 1 (old = 3 per category); 5.2 State 3 (up to 5 results)</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>GS-GRP-02</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1671,17 +1477,8 @@
           <t>requirements.md 5.2 State 3 ('Show all N work orders' link)</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>GS-GRP-03</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1727,17 +1524,8 @@
           <t>requirements.md 5.2 (Show all switches to the scope tab - recommended); Open Question OQ-SPEC-1</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>GS-GRP-04</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1783,17 +1571,8 @@
           <t>requirements.md 6.2 (group display order in 'All')</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>GS-GRP-05</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1839,17 +1618,8 @@
           <t>requirements.md 5.3 (matched substring highlighted)</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>GS-GRP-06</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1895,17 +1665,8 @@
           <t>requirements.md 9 Non-Functional (screen-reader announcements when results count changes; focus rings)</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>GS-GRP-07</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1954,17 +1715,8 @@
           <t>requirements.md 4 Work Orders (Displayed: WO number + customer, status badge, lead technician, asset/unit, date)</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>GS-ENT-01</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2012,17 +1764,8 @@
           <t>requirements.md 4 Customers (Displayed: name, address line, open WO count badge, telephone on hover)</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
-        <is>
-          <t>GS-ENT-02</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2069,17 +1812,8 @@
           <t>requirements.md 4 Assets (Displayed: year + make + model primary, customer name secondary)</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
-        <is>
-          <t>GS-ENT-03</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2128,17 +1862,8 @@
           <t>requirements.md 4 Parts (Displayed: description, part number, total quantity with stock-status color)</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>GS-ENT-04</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2185,17 +1910,8 @@
           <t>requirements.md 4 Vendors (Displayed: vendor name primary, address line secondary)</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>GS-ENT-05</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2243,17 +1959,8 @@
           <t>requirements.md 4 Part Sales (Displayed: P-number + customer primary, status badge, total price + created date)</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
-        <is>
-          <t>GS-ENT-06</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2299,17 +2006,8 @@
           <t>requirements.md 4 (secondary line shows 'Contact/info match')</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>GS-ENT-07</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2355,17 +2053,8 @@
           <t>requirements.md 5.3 (status badge colors, same tokens as the WO list)</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>GS-ENT-08</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2411,17 +2100,8 @@
           <t>requirements.md 7 (token n-gram / trigram matching catches Petersn -&gt; Peterson)</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>GS-FUZ-01</t>
-        </is>
-      </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2466,17 +2146,8 @@
           <t>requirements.md 1 + 10 Phase 5 (fuzzy query 'Abrige')</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>GS-FUZ-02</t>
-        </is>
-      </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2521,17 +2192,8 @@
           <t>requirements.md 7 (Damerau-Levenshtein; freihgtliner -&gt; freightliner)</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>GS-FUZ-03</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2576,17 +2238,8 @@
           <t>requirements.md 7 (phonetic fallback catches Filbridge -&gt; Fibridge)</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>GS-FUZ-04</t>
-        </is>
-      </c>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2634,17 +2287,8 @@
           <t>requirements.md 7 (S2-15276 = s215276); identifier fields are exact-only</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>GS-FUZ-05</t>
-        </is>
-      </c>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2690,17 +2334,8 @@
           <t>requirements.md 7 (What is NOT fuzzy: VIN, WO number, P-number, part number - exact match after normalization)</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>GS-FUZ-06</t>
-        </is>
-      </c>
-      <c r="J40" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2747,17 +2382,8 @@
           <t>requirements.md 7 (phone normalization); 4 (Contact/info match affordance)</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>GS-FUZ-07</t>
-        </is>
-      </c>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2803,17 +2429,8 @@
           <t>requirements.md 7 (What is NOT fuzzy: part number)</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>GS-FUZ-08</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2859,17 +2476,8 @@
           <t>requirements.md 7 (exact identifier fields bypass fuzzy logic)</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t>GS-FUZ-09</t>
-        </is>
-      </c>
-      <c r="J43" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2915,17 +2523,8 @@
           <t>requirements.md 7 (fuzzy soft-match highlight treatment - design polish, confirm with design)</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t>GS-FUZ-10</t>
-        </is>
-      </c>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2971,17 +2570,8 @@
           <t>requirements.md 7 (What is NOT fuzzy: VIN, WO number, P-number, part number - exact match after normalization)</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr">
-        <is>
-          <t>GS-FUZ-11</t>
-        </is>
-      </c>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3027,17 +2617,8 @@
           <t>requirements.md 6.2 (ID match &gt; 0.95 pinned at top)</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>GS-RANK-01</t>
-        </is>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3083,17 +2664,8 @@
           <t>requirements.md 6.1 Work Orders signals (open status +0.30, recency, assigned/viewed, old-closed demoted)</t>
         </is>
       </c>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>GS-RANK-02</t>
-        </is>
-      </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3139,17 +2711,8 @@
           <t>requirements.md 6.1 Parts signals</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>GS-RANK-03</t>
-        </is>
-      </c>
-      <c r="J48" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3195,17 +2758,8 @@
           <t>requirements.md 6.3 Contextual bias</t>
         </is>
       </c>
-      <c r="I49" s="2" t="inlineStr">
-        <is>
-          <t>GS-RANK-04</t>
-        </is>
-      </c>
-      <c r="J49" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K49" s="2" t="inlineStr"/>
+      <c r="I49" s="2" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3251,17 +2805,8 @@
           <t>requirements.md 6.3 Contextual bias</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>GS-RANK-05</t>
-        </is>
-      </c>
-      <c r="J50" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3309,17 +2854,8 @@
           <t>requirements.md 5.2 State 1 (First-time search)</t>
         </is>
       </c>
-      <c r="I51" s="2" t="inlineStr">
-        <is>
-          <t>GS-EMPTY-01</t>
-        </is>
-      </c>
-      <c r="J51" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K51" s="2" t="inlineStr"/>
+      <c r="I51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3367,17 +2903,8 @@
           <t>requirements.md 5.2 State 1 (quick-create chips)</t>
         </is>
       </c>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>GS-EMPTY-02</t>
-        </is>
-      </c>
-      <c r="J52" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K52" s="2" t="inlineStr"/>
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3424,17 +2951,8 @@
           <t>requirements.md 5.2 State 2 (Recent searches grouped by interval); 8 (persist recent-entity-views 30 days)</t>
         </is>
       </c>
-      <c r="I53" s="2" t="inlineStr">
-        <is>
-          <t>GS-REC-01</t>
-        </is>
-      </c>
-      <c r="J53" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K53" s="2" t="inlineStr"/>
+      <c r="I53" s="2" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3481,17 +2999,8 @@
           <t>requirements.md 5.2 State 2 (same row template as a result row)</t>
         </is>
       </c>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>GS-REC-02</t>
-        </is>
-      </c>
-      <c r="J54" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K54" s="2" t="inlineStr"/>
+      <c r="I54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3536,17 +3045,8 @@
           <t>requirements.md 10 Phase 4 (records a touch on every result click / entity-page visit)</t>
         </is>
       </c>
-      <c r="I55" s="2" t="inlineStr">
-        <is>
-          <t>GS-REC-03</t>
-        </is>
-      </c>
-      <c r="J55" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K55" s="2" t="inlineStr"/>
+      <c r="I55" s="2" t="inlineStr"/>
+      <c r="J55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3593,17 +3093,8 @@
           <t>requirements.md 5.2 State 5 (Persisting search); 8 (persist last query, rehydrate on reopen)</t>
         </is>
       </c>
-      <c r="I56" s="2" t="inlineStr">
-        <is>
-          <t>GS-PERS-01</t>
-        </is>
-      </c>
-      <c r="J56" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K56" s="2" t="inlineStr"/>
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3650,17 +3141,8 @@
           <t>requirements.md 5.2 State 5 (Reopening restores the query, the scope tab, and the result list)</t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr">
-        <is>
-          <t>GS-PERS-02</t>
-        </is>
-      </c>
-      <c r="J57" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K57" s="2" t="inlineStr"/>
+      <c r="I57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3706,17 +3188,8 @@
           <t>requirements.md 5.2 State 5; design-notes screenshot 9 (clearable via the x button)</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr">
-        <is>
-          <t>GS-PERS-03</t>
-        </is>
-      </c>
-      <c r="J58" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K58" s="2" t="inlineStr"/>
+      <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3763,17 +3236,8 @@
           <t>requirements.md 5.2 State 4 (No results for &lt;query&gt; + quick-create chips)</t>
         </is>
       </c>
-      <c r="I59" s="2" t="inlineStr">
-        <is>
-          <t>GS-NORES-01</t>
-        </is>
-      </c>
-      <c r="J59" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K59" s="2" t="inlineStr"/>
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3818,17 +3282,8 @@
           <t>requirements.md 5.2 State 4</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr">
-        <is>
-          <t>GS-NORES-02</t>
-        </is>
-      </c>
-      <c r="J60" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3874,17 +3329,8 @@
           <t>requirements.md 5.4 (Work Order -&gt; 'Add new line', only when currently editing a WO elsewhere)</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr">
-        <is>
-          <t>GS-HOVER-01</t>
-        </is>
-      </c>
-      <c r="J61" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K61" s="2" t="inlineStr"/>
+      <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3931,17 +3377,8 @@
           <t>requirements.md 5.4 (Asset -&gt; 'New work order' + clock (history) and Invoice icons)</t>
         </is>
       </c>
-      <c r="I62" s="2" t="inlineStr">
-        <is>
-          <t>GS-HOVER-02</t>
-        </is>
-      </c>
-      <c r="J62" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -3988,17 +3425,8 @@
           <t>requirements.md 5.4 (Customer -&gt; 'New work order', 'New contact')</t>
         </is>
       </c>
-      <c r="I63" s="2" t="inlineStr">
-        <is>
-          <t>GS-HOVER-03</t>
-        </is>
-      </c>
-      <c r="J63" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K63" s="2" t="inlineStr"/>
+      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4045,17 +3473,8 @@
           <t>requirements.md 5.4 (Part -&gt; 'Add part' when not currently editing a WO)</t>
         </is>
       </c>
-      <c r="I64" s="2" t="inlineStr">
-        <is>
-          <t>GS-HOVER-04</t>
-        </is>
-      </c>
-      <c r="J64" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4101,17 +3520,8 @@
           <t>requirements.md 5.4 (Vendor -&gt; 'Add contact')</t>
         </is>
       </c>
-      <c r="I65" s="2" t="inlineStr">
-        <is>
-          <t>GS-HOVER-05</t>
-        </is>
-      </c>
-      <c r="J65" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K65" s="2" t="inlineStr"/>
+      <c r="I65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4158,17 +3568,8 @@
           <t>requirements.md 5.4 (Part -&gt; 'Add to work order' only when currently editing a WO)</t>
         </is>
       </c>
-      <c r="I66" s="2" t="inlineStr">
-        <is>
-          <t>GS-HOVER-06</t>
-        </is>
-      </c>
-      <c r="J66" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K66" s="2" t="inlineStr"/>
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -4213,17 +3614,8 @@
           <t>requirements.md 5.4 (Quick actions never trigger destructive operations; hover state non-essential)</t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr">
-        <is>
-          <t>GS-HOVER-07</t>
-        </is>
-      </c>
-      <c r="J67" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K67" s="2" t="inlineStr"/>
+      <c r="I67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -4271,17 +3663,8 @@
           <t>design-notes screenshot 1 (in-page Work Orders list search banner)</t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr">
-        <is>
-          <t>GS-LIST-01</t>
-        </is>
-      </c>
-      <c r="J68" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K68" s="2" t="inlineStr"/>
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4326,17 +3709,8 @@
           <t>design-notes screenshot 1</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr">
-        <is>
-          <t>GS-LIST-02</t>
-        </is>
-      </c>
-      <c r="J69" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K69" s="2" t="inlineStr"/>
+      <c r="I69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4384,17 +3758,8 @@
           <t>requirements.md 8 (tolerate offline/network failures with an inline 'Search unavailable, retry' banner)</t>
         </is>
       </c>
-      <c r="I70" s="2" t="inlineStr">
-        <is>
-          <t>GS-ERR-01</t>
-        </is>
-      </c>
-      <c r="J70" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K70" s="2" t="inlineStr"/>
+      <c r="I70" s="2" t="inlineStr"/>
+      <c r="J70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4440,17 +3805,8 @@
           <t>requirements.md 9 (all result fields respect role-based-access checks)</t>
         </is>
       </c>
-      <c r="I71" s="2" t="inlineStr">
-        <is>
-          <t>GS-PERM-01</t>
-        </is>
-      </c>
-      <c r="J71" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K71" s="2" t="inlineStr"/>
+      <c r="I71" s="2" t="inlineStr"/>
+      <c r="J71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4497,17 +3853,8 @@
           <t>requirements.md 9 (a technician without Parts access does not see Parts results)</t>
         </is>
       </c>
-      <c r="I72" s="2" t="inlineStr">
-        <is>
-          <t>GS-PERM-02</t>
-        </is>
-      </c>
-      <c r="J72" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K72" s="2" t="inlineStr"/>
+      <c r="I72" s="2" t="inlineStr"/>
+      <c r="J72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4553,17 +3900,8 @@
           <t>requirements.md 9 (all result fields respect role-based-access checks)</t>
         </is>
       </c>
-      <c r="I73" s="2" t="inlineStr">
-        <is>
-          <t>GS-PERM-03</t>
-        </is>
-      </c>
-      <c r="J73" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K73" s="2" t="inlineStr"/>
+      <c r="I73" s="2" t="inlineStr"/>
+      <c r="J73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4609,17 +3947,8 @@
           <t>requirements.md 9 (all result fields respect existing tenant-isolation checks)</t>
         </is>
       </c>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>GS-PERM-04</t>
-        </is>
-      </c>
-      <c r="J74" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K74" s="2" t="inlineStr"/>
+      <c r="I74" s="2" t="inlineStr"/>
+      <c r="J74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4667,17 +3996,8 @@
           <t>requirements.md 9 (must work for a single-tenant dataset where any entity type is empty, e.g. no part sales yet)</t>
         </is>
       </c>
-      <c r="I75" s="2" t="inlineStr">
-        <is>
-          <t>GS-PERM-05</t>
-        </is>
-      </c>
-      <c r="J75" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K75" s="2" t="inlineStr"/>
+      <c r="I75" s="2" t="inlineStr"/>
+      <c r="J75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4724,17 +4044,8 @@
           <t>requirements.md 10 Phase 1 (GET /api/search; scope=all)</t>
         </is>
       </c>
-      <c r="I76" s="2" t="inlineStr">
-        <is>
-          <t>GS-API-01</t>
-        </is>
-      </c>
-      <c r="J76" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K76" s="2" t="inlineStr"/>
+      <c r="I76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -4782,17 +4093,8 @@
           <t>requirements.md 10 Phase 1 (scope parameter)</t>
         </is>
       </c>
-      <c r="I77" s="2" t="inlineStr">
-        <is>
-          <t>GS-API-02</t>
-        </is>
-      </c>
-      <c r="J77" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K77" s="2" t="inlineStr"/>
+      <c r="I77" s="2" t="inlineStr"/>
+      <c r="J77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -4840,17 +4142,8 @@
           <t>requirements.md 10 Phase 1 (limit default 5; response includes per-group totals)</t>
         </is>
       </c>
-      <c r="I78" s="2" t="inlineStr">
-        <is>
-          <t>GS-API-03</t>
-        </is>
-      </c>
-      <c r="J78" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K78" s="2" t="inlineStr"/>
+      <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -4899,17 +4192,8 @@
           <t>requirements.md 7 (identifier normalization); 6.2 (ID match pinned)</t>
         </is>
       </c>
-      <c r="I79" s="2" t="inlineStr">
-        <is>
-          <t>GS-API-04</t>
-        </is>
-      </c>
-      <c r="J79" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K79" s="2" t="inlineStr"/>
+      <c r="I79" s="2" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -4955,17 +4239,8 @@
           <t>requirements.md 7 (What is NOT fuzzy)</t>
         </is>
       </c>
-      <c r="I80" s="2" t="inlineStr">
-        <is>
-          <t>GS-API-05</t>
-        </is>
-      </c>
-      <c r="J80" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K80" s="2" t="inlineStr"/>
+      <c r="I80" s="2" t="inlineStr"/>
+      <c r="J80" s="2" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -5013,17 +4288,8 @@
           <t>requirements.md 9 (results respect role-based-access checks - enforced server-side)</t>
         </is>
       </c>
-      <c r="I81" s="2" t="inlineStr">
-        <is>
-          <t>GS-API-06</t>
-        </is>
-      </c>
-      <c r="J81" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K81" s="2" t="inlineStr"/>
+      <c r="I81" s="2" t="inlineStr"/>
+      <c r="J81" s="2" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -5071,17 +4337,8 @@
           <t>requirements.md 8 (offline/network failure handling)</t>
         </is>
       </c>
-      <c r="I82" s="2" t="inlineStr">
-        <is>
-          <t>GS-API-07</t>
-        </is>
-      </c>
-      <c r="J82" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K82" s="2" t="inlineStr"/>
+      <c r="I82" s="2" t="inlineStr"/>
+      <c r="J82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -5128,17 +4385,8 @@
           <t>requirements.md 6.2 (group order); 10 Phase 1 (per-item metadata)</t>
         </is>
       </c>
-      <c r="I83" s="2" t="inlineStr">
-        <is>
-          <t>GS-API-08</t>
-        </is>
-      </c>
-      <c r="J83" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K83" s="2" t="inlineStr"/>
+      <c r="I83" s="2" t="inlineStr"/>
+      <c r="J83" s="2" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -5186,17 +4434,8 @@
           <t>requirements.md 10 Phase 1 (cursor parameter)</t>
         </is>
       </c>
-      <c r="I84" s="2" t="inlineStr">
-        <is>
-          <t>GS-API-09</t>
-        </is>
-      </c>
-      <c r="J84" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K84" s="2" t="inlineStr"/>
+      <c r="I84" s="2" t="inlineStr"/>
+      <c r="J84" s="2" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -5243,17 +4482,8 @@
           <t>requirements.md 6.3 (contextual bias); 10 Phase 1 (context parameter)</t>
         </is>
       </c>
-      <c r="I85" s="2" t="inlineStr">
-        <is>
-          <t>GS-API-10</t>
-        </is>
-      </c>
-      <c r="J85" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K85" s="2" t="inlineStr"/>
+      <c r="I85" s="2" t="inlineStr"/>
+      <c r="J85" s="2" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -5300,17 +4530,8 @@
           <t>requirements.md 8 (persist recent-entity-views 30 days); 10 Phase 4</t>
         </is>
       </c>
-      <c r="I86" s="2" t="inlineStr">
-        <is>
-          <t>GS-API-11</t>
-        </is>
-      </c>
-      <c r="J86" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K86" s="2" t="inlineStr"/>
+      <c r="I86" s="2" t="inlineStr"/>
+      <c r="J86" s="2" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -5357,17 +4578,8 @@
           <t>requirements.md 8 (debounce input at 150ms; render within 200ms p95)</t>
         </is>
       </c>
-      <c r="I87" s="2" t="inlineStr">
-        <is>
-          <t>GS-API-12</t>
-        </is>
-      </c>
-      <c r="J87" s="2" t="inlineStr">
-        <is>
-          <t>pending push</t>
-        </is>
-      </c>
-      <c r="K87" s="2" t="inlineStr"/>
+      <c r="I87" s="2" t="inlineStr"/>
+      <c r="J87" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Global Search: v2 content update in place (no removals) — placeholder(no-AI), inventory not catalogue, 9-entity tabs/group order (D16), tabs-only replacing Show-all; suite stays 97/97 compliant
</commit_message>
<xml_diff>
--- a/testrail-import/global-search-v2-testrail-import.xlsx
+++ b/testrail-import/global-search-v2-testrail-import.xlsx
@@ -676,15 +676,33 @@
 a
 d
 s
+a
+p
+l
+a
+i
+n
+s
+e
+a
+r
+c
+h
+p
+l
+a
+c
+e
+h
+o
+l
+d
+e
+r
+(
+n
+o
 '
-S
-e
-a
-r
-c
-h
-o
-r
 a
 s
 k
@@ -698,6 +716,45 @@
 o
 n
 '
+/
+A
+I
+w
+o
+r
+d
+i
+n
+g
+i
+n
+v
+1
+-
+e
+x
+a
+c
+t
+c
+o
+p
+y
+p
+e
+r
+t
+h
+e
+v
+2
+d
+e
+s
+i
+g
+n
+)
 .
 5
 .
@@ -1228,15 +1285,33 @@
 d
 e
 r
+a
+p
+l
+a
+i
+n
+s
+e
+a
+r
+c
+h
+p
+l
+a
+c
+e
+h
+o
+l
+d
+e
+r
+(
+n
+o
 '
-S
-e
-a
-r
-c
-h
-o
-r
 a
 s
 k
@@ -1250,6 +1325,45 @@
 o
 n
 '
+/
+A
+I
+w
+o
+r
+d
+i
+n
+g
+i
+n
+v
+1
+-
+e
+x
+a
+c
+t
+c
+o
+p
+y
+p
+e
+r
+t
+h
+e
+v
+2
+d
+e
+s
+i
+g
+n
+)
 .
 4
 .
@@ -5199,6 +5313,15 @@
 r
 s
 ,
+C
+o
+n
+t
+a
+c
+t
+s
+,
 A
 s
 s
@@ -5229,6 +5352,56 @@
 l
 e
 s
+,
+P
+u
+r
+c
+h
+a
+s
+e
+O
+r
+d
+e
+r
+s
+,
+V
+e
+n
+d
+o
+r
+I
+n
+v
+o
+i
+c
+e
+s
+(
+v
+2
+n
+i
+n
+e
+e
+n
+t
+i
+t
+i
+e
+s
+,
+D
+1
+6
+)
 .
 2
 .
@@ -5262,6 +5435,83 @@
 u
 l
 t
+.
+3
+.
+A
+t
+a
+b
+i
+s
+s
+h
+o
+w
+n
+o
+n
+l
+y
+f
+o
+r
+a
+n
+e
+n
+t
+i
+t
+y
+t
+y
+p
+e
+t
+h
+e
+u
+s
+e
+r
+h
+a
+s
+p
+e
+r
+m
+i
+s
+s
+i
+o
+n
+t
+o
+s
+e
+e
+(
+p
+e
+r
+m
+i
+s
+s
+i
+o
+n
+-
+s
+c
+o
+p
+e
+d
+)
 .
 -
 -
@@ -5629,6 +5879,10 @@
 t
 h
 a
+t
+r
+u
+e
 c
 o
 u
@@ -5650,7 +5904,7 @@
 o
 r
 k
-o
+O
 r
 d
 e
@@ -5697,11 +5951,25 @@
 t
 h
 e
-o
-r
-d
-e
-r
+v
+2
+n
+i
+n
+e
+-
+e
+n
+t
+i
+t
+y
+o
+r
+d
+e
+r
+:
 W
 o
 r
@@ -5723,6 +5991,15 @@
 r
 s
 ,
+C
+o
+n
+t
+a
+c
+t
+s
+,
 A
 s
 s
@@ -5753,6 +6030,41 @@
 l
 e
 s
+,
+P
+u
+r
+c
+h
+a
+s
+e
+O
+r
+d
+e
+r
+s
+,
+V
+e
+n
+d
+o
+r
+I
+n
+v
+o
+i
+c
+e
+s
+(
+D
+1
+6
+)
 .
 -
 -
@@ -10113,50 +10425,15 @@
         <is>
           <t xml:space="preserve">1
 .
-A
-l
-i
-n
-k
-a
-p
-p
-e
-a
-r
-s
-a
-t
-t
-h
-e
-b
-o
-t
-t
-o
-m
-o
-f
-t
-h
-e
-g
-r
-o
-u
-p
-,
-w
-o
-r
-d
-e
-d
-l
-i
-k
-e
+T
+h
+e
+r
+e
+i
+s
+N
+O
 '
 S
 h
@@ -10165,102 +10442,200 @@
 a
 l
 l
+N
+'
+l
+i
+n
+k
+i
+n
+v
+2
+(
+d
+r
+o
+p
+p
+e
+d
+b
+y
+D
+1
+5
+/
+F
+R
+-
+0
+1
+3
+)
+.
+2
+.
+I
+n
+t
+h
+e
+A
+l
+l
+v
+i
+e
 w
+a
+g
+r
+o
+u
+p
+s
+h
+o
+w
+s
+u
+p
+t
+o
+5
+r
+o
+w
+s
+w
+i
+t
+h
+i
+t
+s
+t
+r
+u
+e
+t
+o
+t
+a
+l
+i
+n
+t
+h
+e
+h
+e
+a
+d
+i
+n
+g
+(
+f
+o
+r
+e
+x
+a
+m
+p
+l
+e
+'
+W
 o
 r
 k
-o
-r
-d
-e
-r
-s
-'
+O
+r
+d
+e
+r
+s
 (
-o
-r
-'
-S
-h
-o
-w
-a
-l
-l
-1
-2
-w
-o
-r
-k
-o
-r
-d
-e
-r
-s
+1
+2
+)
 '
 )
 .
-2
+3
 .
 T
-h
-e
-l
-i
-n
-k
-o
-n
-l
+o
+s
+e
+e
+m
+o
+r
+e
+t
+h
+a
+n
+5
+,
+t
+h
+e
+u
+s
+e
+r
+o
+p
+e
+n
+s
+t
+h
+a
+t
+e
+n
+t
+i
+t
 y
-a
-p
-p
-e
-a
-r
-s
-w
-h
-e
-n
-t
-h
-e
-r
-e
-a
-r
-e
-m
-o
-r
-e
-m
-a
-t
-c
-h
-e
-s
-t
-h
-a
-n
-t
-h
-e
-r
-o
-w
-s
-s
-h
-o
-w
-n
+'
+s
+s
+c
+o
+p
+e
+t
+a
+b
+(
+s
+e
+e
+t
+h
+e
+S
+c
+o
+p
+e
+T
+a
+b
+s
+c
+a
+s
+e
+s
+)
 .
 -
 -
@@ -10541,239 +10916,240 @@
         <is>
           <t xml:space="preserve">1
 .
+O
+p
+e
+n
+i
+n
+g
+a
+n
+e
+n
+t
+i
+t
+y
+'
+s
+s
+c
+o
+p
+e
+t
+a
+b
+(
+n
+o
+t
+a
+'
+S
+h
+o
+w
+a
+l
+l
+'
+l
+i
+n
+k
+,
+w
+h
+i
+c
+h
+n
+o
+l
+o
+n
+g
+e
+r
+e
+x
+i
+s
+t
+s
+)
+s
+h
+o
+w
+s
+t
+h
+a
+t
+e
+n
+t
+i
+t
+y
+'
+s
+f
+u
+l
+l
+r
+e
+s
+u
+l
+t
+l
+i
+s
+t
+w
+i
+t
+h
+i
+n
+t
+h
+e
+m
+o
+d
+a
+l
+.
+2
+.
 T
 h
 e
-p
-a
-l
-e
-t
-t
-e
-s
-t
+s
+c
+o
+p
+e
+d
+l
+i
+s
+t
+l
+o
+a
+d
+s
+a
+d
+e
+f
+a
+u
+l
+t
+p
+a
+g
+e
+(
+2
+5
+)
+w
+i
+t
+h
+c
+u
+r
+s
+o
+r
+-
+b
+a
+s
+e
+d
+l
+o
+a
+d
+-
+m
+o
+r
+e
+i
+n
+s
+i
+d
+e
+t
+h
+e
+m
+o
+d
+a
+l
+.
+3
+.
+T
+h
+e
+m
+o
+d
+a
+l
+d
+o
+e
+s
+n
+o
+t
+n
+a
+v
+i
+g
+a
+t
+e
+a
+w
 a
 y
-s
-o
-p
-e
-n
-a
-n
-d
-s
-w
-i
-t
-c
-h
-e
-s
-t
-o
-t
-h
-e
-'
-W
-o
-r
-k
-O
-r
-d
-e
-r
-s
-'
-s
-c
-o
-p
-e
-t
-a
-b
-.
-2
-.
-T
-h
+t
+o
+a
+s
+e
+p
+a
+r
+a
+t
 e
 f
 u
 l
 l
-l
-i
-s
-t
-o
-f
-m
-a
-t
-c
-h
-i
-n
-g
-W
-o
-r
-k
-O
-r
-d
-e
-r
-s
-f
-o
-r
-t
-h
-e
-c
-u
-r
-r
-e
-n
-t
-q
-u
-e
-r
-y
-i
-s
-s
-h
-o
-w
-n
-,
-s
-c
-o
-p
-e
-d
-t
-o
-W
-o
-r
-k
-O
-r
-d
-e
-r
-s
-o
-n
-l
-y
-.
-3
-.
-T
-h
-e
-p
-a
-l
-e
-t
-t
-e
-d
-o
-e
-s
-n
-o
-t
-l
-e
-a
-v
-e
-t
-o
-a
-s
-e
-p
-a
-r
-a
-t
-e
-f
-u
-l
-l
-p
-a
-g
-e
-(
-t
-h
-e
-r
-e
-c
-o
-m
-m
-e
-n
-d
-e
-d
-b
-e
-h
-a
-v
-i
-o
-r
-i
-s
-t
-h
-e
-s
-c
-o
-p
-e
-d
-t
-a
-b
-w
-i
-t
-h
-i
-n
-t
-h
-e
-m
-o
-d
-a
-l
-)
+p
+a
+g
+e
 .
 -
 -
@@ -11119,6 +11495,19 @@
 h
 i
 s
+v
+2
+n
+i
+n
+e
+-
+e
+n
+t
+i
+t
+y
 o
 r
 d
@@ -11146,6 +11535,15 @@
 r
 s
 ,
+C
+o
+n
+t
+a
+c
+t
+s
+,
 A
 s
 s
@@ -11176,6 +11574,41 @@
 l
 e
 s
+,
+P
+u
+r
+c
+h
+a
+s
+e
+O
+r
+d
+e
+r
+s
+,
+V
+e
+n
+d
+o
+r
+I
+n
+v
+o
+i
+c
+e
+s
+(
+D
+1
+6
+)
 .
 2
 .
@@ -24695,15 +25128,33 @@
 d
 e
 r
+a
+p
+l
+a
+i
+n
+s
+e
+a
+r
+c
+h
+p
+l
+a
+c
+e
+h
+o
+l
+d
+e
+r
+(
+n
+o
 '
-S
-e
-a
-r
-c
-h
-o
-r
 a
 s
 k
@@ -24717,6 +25168,45 @@
 o
 n
 '
+/
+A
+I
+w
+o
+r
+d
+i
+n
+g
+i
+n
+v
+1
+-
+e
+x
+a
+c
+t
+c
+o
+p
+y
+p
+e
+r
+t
+h
+e
+v
+2
+d
+e
+s
+i
+g
+n
+)
 .
 2
 .
@@ -29366,15 +29856,33 @@
 d
 e
 r
+a
+p
+l
+a
+i
+n
+s
+e
+a
+r
+c
+h
+p
+l
+a
+c
+e
+h
+o
+l
+d
+e
+r
+(
+n
+o
 '
-S
-e
-a
-r
-c
-h
-o
-r
 a
 s
 k
@@ -29388,6 +29896,45 @@
 o
 n
 '
+/
+A
+I
+w
+o
+r
+d
+i
+n
+g
+i
+n
+v
+1
+-
+e
+x
+a
+c
+t
+c
+o
+p
+y
+p
+e
+r
+t
+h
+e
+v
+2
+d
+e
+s
+i
+g
+n
+)
 )
 .
 3
@@ -31825,9 +32372,100 @@
         <is>
           <t xml:space="preserve">1
 .
+O
+n
+h
+o
+v
+e
+r
+a
+P
+a
+r
+t
+q
+u
+i
+c
+k
+a
+c
+t
+i
+o
+n
+a
+p
+p
+e
+a
+r
+s
+:
+"
 A
-n
-'
+d
+d
+t
+o
+w
+o
+r
+k
+o
+r
+d
+e
+r
+"
+w
+h
+e
+n
+y
+o
+u
+a
+r
+e
+c
+u
+r
+r
+e
+n
+t
+l
+y
+e
+d
+i
+t
+i
+n
+g
+a
+w
+o
+r
+k
+o
+r
+d
+e
+r
+,
+o
+t
+h
+e
+r
+w
+i
+s
+e
+"
 A
 d
 d
@@ -31835,29 +32473,59 @@
 a
 r
 t
-'
-b
-u
-t
-t
-o
-n
-a
-p
-p
-e
-a
-r
-s
-o
-n
-h
-o
+"
+.
+2
+.
+T
+h
+e
+P
+a
+r
+t
+r
+o
+w
+n
+a
 v
-e
-r
-.
-2
+i
+g
+a
+t
+e
+s
+t
+o
+I
+N
+V
+E
+N
+T
+O
+R
+Y
+(
+n
+o
+t
+t
+h
+e
+c
+a
+t
+a
+l
+o
+g
+u
+e
+)
+.
+3
 .
 T
 h
@@ -43096,11 +43764,25 @@
 t
 h
 e
-o
-r
-d
-e
-r
+v
+2
+n
+i
+n
+e
+-
+e
+n
+t
+i
+t
+y
+o
+r
+d
+e
+r
+:
 W
 o
 r
@@ -43122,6 +43804,15 @@
 r
 s
 ,
+C
+o
+n
+t
+a
+c
+t
+s
+,
 A
 s
 s
@@ -43152,6 +43843,41 @@
 l
 e
 s
+,
+P
+u
+r
+c
+h
+a
+s
+e
+O
+r
+d
+e
+r
+s
+,
+V
+e
+n
+d
+o
+r
+I
+n
+v
+o
+i
+c
+e
+s
+(
+D
+1
+6
+)
 .
 2
 .
@@ -43202,6 +43928,25 @@
 i
 n
 g
+;
+t
+i
+e
+s
+b
+r
+e
+a
+k
+b
+y
+r
+e
+c
+e
+n
+c
+y
 .
 3
 .
@@ -43287,11 +44032,11 @@
 d
 s
 ,
-s
-t
-a
-t
-u
+b
+a
+d
+g
+e
 s
 /
 q
@@ -43327,6 +44072,29 @@
 c
 h
 e
+s
+,
+a
+n
+d
+t
+r
+u
+e
+p
+e
+r
+-
+g
+r
+o
+u
+p
+t
+o
+t
+a
+l
 s
 .
 -

</xml_diff>

<commit_message>
Global Search: resolve PO-GS-5/6 defensively (110 cases)
PO-GS-5: telemetry IS v1 per PRD section 8 (functional) + 6.4 - added GS-TEL-01
with a scope note (SV-9167 backlogged; if absent on build, raise as deviation,
never silently pass). PO-GS-6: GS-VI-01 kept Paid/Unpaid per section 5.3 but made
tolerant of a third 'Partially paid' state as a documented known-variance, not a
failure. Both PO questions stay open for Branko; cases can't bite a tester either way.
Regenerated import (110) + id-map.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QvLHRX1rY5c7HuyoMWVGpU
</commit_message>
<xml_diff>
--- a/testrail-import/global-search-v2-testrail-import.xlsx
+++ b/testrail-import/global-search-v2-testrail-import.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J110"/>
+  <dimension ref="A1:J111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -4002,7 +4002,7 @@
       <c r="G71" s="2" t="inlineStr">
         <is>
           <t>1. The Work Orders list filters to only rows matching 'Fib'.
-2. A blue banner reads 'Showing 12 work orders matching \'Fib\'' (the count reflects the number of matches).
+2. A blue banner reads 'Showing 12 work orders matching "Fib"' (the count reflects the number of matches).
 3. A 'Clear search' link appears on the right of the banner.
 4. The list columns remain: On Site, Status, Number, Customer, Asset, Unit, VIN/Serial #, Progress, Service Advisor, Lead Technician, Clocked In, Lines, Total Price.
 ---
@@ -5964,53 +5964,106 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
+          <t>Search impressions and clicks are recorded (search-event telemetry)</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Search Telemetry</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>The global search palette is available and returns results.</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>Run a query so results are shown (impressions).
+Click a result.
+Have engineering/QA confirm the search-event log.</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>1. Each result impression is logged with the query, result entity type, result id and position.
+2. A click on a result is logged as was_clicked for that result.
+3. This is mechanism/schema only - no ML ranking model is expected in v1.
+4. SCOPE NOTE (PO-GS-5): the owning story SV-9167 is currently in the backlog. If event logging is not present on the build, record it as a deviation to raise with Product - do not silently pass or ignore it.
+---
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 8 (functional requirements) / 6.4 (telemetry schema), read on 25 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>section 8 / 6.4 (telemetry)</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr"/>
+      <c r="J110" s="2" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
           <t>Vendor Invoices searchable; tri-state payment badge; no quick action</t>
         </is>
       </c>
-      <c r="B110" s="2" t="inlineStr">
+      <c r="B111" s="2" t="inlineStr">
         <is>
           <t>Vendor Invoices Entity (v2)</t>
         </is>
       </c>
-      <c r="C110" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D110" s="2" t="inlineStr">
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E110" s="2" t="inlineStr">
+      <c r="E111" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in with Vendor &amp; Order Management access.
 2. Vendor invoices exist in unpaid, partially paid and paid states.</t>
         </is>
       </c>
-      <c r="F110" s="2" t="inlineStr">
+      <c r="F111" s="2" t="inlineStr">
         <is>
           <t>1. Open global search and search for a vendor invoice.
 2. Look at the Vendor Invoices group, the row and its payment badge.</t>
         </is>
       </c>
-      <c r="G110" s="2" t="inlineStr">
+      <c r="G111" s="2" t="inlineStr">
         <is>
           <t>1. Vendor Invoices appear as their own searchable entity, grouped under a 'Vendor Invoices' heading with a true count and a scope tab (subject to permission).
-2. A vendor-invoice row carries the file-text icon; the primary line shows the invoice number + vendor, with a status badge (Paid / Unpaid), the total, the invoice date, and the type (Invoice / Sublet).
-3. Vendor Invoice results are gated by Vendor &amp; Order Management: View, and the invoice total is masked for a user without See Financial Data.
+2. A vendor-invoice row carries the file-text icon; the primary line shows the invoice number + vendor, with the total, the invoice date, and the type (Invoice / Sublet).
+3. The payment status badge per the spec (section 5.3) is Paid or Unpaid. KNOWN VARIANCE (PO-GS-6): if the build shows a third 'Partially paid' state, treat it as an expected variance to confirm with Product - do NOT fail the case on it.
+4. Vendor Invoice results are gated by Vendor &amp; Order Management: View, and the invoice total is masked for a user without See Financial Data.
 ---
 This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.3 / 6.1 (Vendor Invoices row), read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
-      <c r="H110" s="2" t="inlineStr">
+      <c r="H111" s="2" t="inlineStr">
         <is>
           <t>section 5.3 / 6.1 (Vendor Invoices row)</t>
         </is>
       </c>
-      <c r="I110" s="2" t="inlineStr"/>
-      <c r="J110" s="2" t="inlineStr"/>
+      <c r="I111" s="2" t="inlineStr"/>
+      <c r="J111" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Global Search: source-verify 110 functional cases to PRD v12 (re-pin; no content change)
PRD moved Confluence v11 -> v12 (unlogged; in-body still 1.2). Full two-fetch
comparison: only content change is section 4 Work Orders 'Indexed' dropping
'status'. Grep-confirmed no functional case searches a WO by status, so no case
content changed. Re-pinned all 110 provenance stamps v11 -> v12 (read 26 Aug),
locally and in TestRail (update_case on all 110, lossless). WO-status drop kept
as PO-REG-6. v12 note saved; requirements marker added.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QvLHRX1rY5c7HuyoMWVGpU
</commit_message>
<xml_diff>
--- a/testrail-import/global-search-v2-testrail-import.xlsx
+++ b/testrail-import/global-search-v2-testrail-import.xlsx
@@ -529,7 +529,7 @@
 4. The placeholder reads a plain search placeholder (no 'ask a question' / AI wording in v1 - exact copy per the v2 design).
 5. The footer keyboard legend is visible: 'Navigate' with up/down arrows, 'Select' with the enter symbol, and 'Close esc'.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.1 Trigger and Surface; 8 Functional Requirements, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.1 Trigger and Surface; 8 Functional Requirements, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -581,7 +581,7 @@
 3. The input is focused and shows the placeholder a plain search placeholder (no 'ask a question' / AI wording in v1 - exact copy per the v2 design).
 4. The footer keyboard legend is visible.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.1 Trigger and Surface, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.1 Trigger and Surface, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -631,7 +631,7 @@
 2. The dimming is removed and you are back on the page you were on.
 3. Keyboard focus returns to the page (or the header search field).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.1; 5.5 Keyboard Navigation, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.1; 5.5 Keyboard Navigation, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -680,7 +680,7 @@
           <t>1. The search box closes.
 2. The dimming is removed and you are back on the page.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.1 (Esc, clicking underlay, or Cmd+K again closes it), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.1 (Esc, clicking underlay, or Cmd+K again closes it), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -730,7 +730,7 @@
           <t>1. The search box closes.
 2. The dimming is removed and you are back on the page.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.1 (clicking the page underlay closes it), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.1 (clicking the page underlay closes it), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -783,7 +783,7 @@
 3. The highlight moves only across result rows - the group heading lines (for example 'Work orders (12)') are skipped and never get the highlight.
 4. When moving down past the last row of one group, the highlight continues into the first row of the next group.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.5 (Up/Down moves focus through visible rows, skipping group headers), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.5 (Up/Down moves focus through visible rows, skipping group headers), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -833,7 +833,7 @@
           <t>1. The palette closes and the highlighted record opens in the same browser tab.
 2. You land on that record's page (for example the Work Order detail page).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.5 (Enter opens the focused row in the same tab), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.5 (Enter opens the focused row in the same tab), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -883,7 +883,7 @@
           <t>1. The highlighted record opens in a NEW browser tab.
 2. The page you were on (and, per build behavior, the palette) remains in the original tab.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.5 (Cmd+Enter or Ctrl+Enter opens in a new browser tab), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.5 (Cmd+Enter or Ctrl+Enter opens in a new browser tab), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -937,7 +937,7 @@
 3. Selecting a tab scopes the results to that entity type.
 4. Focus does not leave the palette (focus stays trapped inside the modal).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.5 (Tab moves focus to the scope tab strip; Left/Right cycles tabs when focus is on the tab strip), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.5 (Tab moves focus to the scope tab strip; Left/Right cycles tabs when focus is on the tab strip), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -987,7 +987,7 @@
           <t>1. The footer keyboard legend is visible in every state: 'Navigate' with up/down arrows, 'Select' with the enter symbol, and 'Close esc'.
 2. The legend does not disappear when results are showing or when the input is empty.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.1 (footer always shows the keyboard legend), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.1 (footer always shows the keyboard legend), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1038,7 +1038,7 @@
 4. The strip scrolls horizontally since ten tabs do not fit the 640px modal width.
 5. A tab is shown only for an entity type the user has permission to see.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 (tab strip), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 (tab strip), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1089,7 +1089,7 @@
           <t>1. Results from every matching entity type appear, each under its own group heading with a true count (for example 'Work Orders (12)', 'Customers (2)').
 2. Groups appear in the v2 nine-entity order: Work Orders, Customers, Contacts, Assets, Parts, Vendors, Part Sales, Purchase Orders, Vendor Invoices (D16).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 State 3; 6.2 group order, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 State 3; 6.2 group order, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1138,7 +1138,7 @@
           <t>1. Only Work Order results are shown; other entity groups (Customers, Assets, Parts, Vendors, Part Sales) are hidden.
 2. The 'Work Orders' tab appears selected/active.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 State 3 (selecting a tab scopes the query to that entity type), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 State 3 (selecting a tab scopes the query to that entity type), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1187,7 +1187,7 @@
           <t>1. Only Customer results are shown; other entity groups are hidden.
 2. The 'Customers' tab appears selected/active.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 State 3, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 State 3, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1236,7 +1236,7 @@
           <t>1. Only Asset results are shown; other entity groups are hidden.
 2. The 'Assets' tab appears selected/active.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 State 3, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 State 3, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1285,7 +1285,7 @@
           <t>1. Only Part results are shown; other entity groups are hidden.
 2. The 'Parts' tab appears selected/active.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 State 3, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 State 3, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1334,7 +1334,7 @@
           <t>1. Only Vendor results are shown; other entity groups are hidden.
 2. The 'Vendors' tab appears selected/active.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 State 3, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 State 3, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1384,7 +1384,7 @@
           <t>1. Only Part Sales results are shown; other entity groups are hidden.
 2. The 'Part Sales' tab appears selected/active.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 4 (Part Sales is a NEW searchable entity); 5.2 State 3, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 4 (Part Sales is a NEW searchable entity); 5.2 State 3, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1437,7 +1437,7 @@
 2. Within the scoped tab the results carry that entity's true total count in the heading.
 3. When the scoped entity has more than five matches the same 'Show all N' link is available (full-page handoff per the Show-all case).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 (scope tab scoping), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 (scope tab scoping), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1485,7 +1485,7 @@
           <t>1. Selecting the 'Contacts' tab scopes the query to contacts only.
 2. The tab carries the true contact count; results show contact rows only.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), 5.2 (Contacts scope tab), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), 5.2 (Contacts scope tab), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1533,7 +1533,7 @@
           <t>1. Selecting the 'Purchase Orders' tab scopes the query to purchase orders only.
 2. The tab carries the true PO count; results show PO rows only (subject to permission).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), 5.2 (Purchase Orders scope tab), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), 5.2 (Purchase Orders scope tab), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1581,7 +1581,7 @@
           <t>1. Selecting the 'Vendor Invoices' tab scopes the query to vendor invoices only.
 2. The tab carries the true count; results show vendor-invoice rows only (subject to permission).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), 5.2 (Vendor Invoices scope tab), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), 5.2 (Vendor Invoices scope tab), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1631,7 +1631,7 @@
           <t>1. Each group heading shows the entity name and the total count in parentheses, for example 'Work orders (12)' and 'Customers (2)'.
 2. The count reflects the total number of matches for that entity type, even when only the first few rows are shown.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 State 3 (results grouped by entity type with a count), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 State 3 (results grouped by entity type with a count), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1681,7 +1681,7 @@
           <t>1. The group shows at most five result rows.
 2. It does not show six or more rows inline (the old behavior was three - it is now five).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 1 (old = 3 per category); 5.2 State 3 (up to 5 results), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 1 (old = 3 per category); 5.2 State 3 (up to 5 results), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1732,7 +1732,7 @@
 2. A group with five or fewer matches shows no 'Show all' link.
 3. The number N reflects the true total for that entity in the current query, not the capped five.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 (Show all N link), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 (Show all N link), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1784,7 +1784,7 @@
 4. While the handoff filter is active, the list page's own inline search field stays empty so the two filters are not confused.
 5. This is implemented for Work Orders in the prototype; each remaining entity list is expected to get the same treatment.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 (Show all - full-page handoff and results banner), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 (Show all - full-page handoff and results banner), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1834,7 +1834,7 @@
           <t>1. The groups appear top to bottom in this v2 nine-entity order: Work Orders, Customers, Contacts, Assets, Parts, Vendors, Part Sales, Purchase Orders, Vendor Invoices (D16).
 2. The order does not change based on how many matches each group has.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 6.2 (group display order in 'All'), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 6.2 (group display order in 'All'), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1884,7 +1884,7 @@
           <t>1. The matched substring 'Fib' is visually highlighted (in the captures it is highlighted in yellow) inside the result's primary text.
 2. Only the matched portion is highlighted, not the whole row.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.3 (matched substring highlighted), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.3 (matched substring highlighted), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1934,7 +1934,7 @@
           <t>1. The screen reader announces the total results count when it changes, for example 'X results found across N categories'.
 2. Every interactive element (input, tabs, rows, links) has a visible focus ring when reached by keyboard.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 9 Non-Functional (screen-reader announcements when results count changes; focus rings), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 9 Non-Functional (screen-reader announcements when results count changes; focus rings), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -1985,7 +1985,7 @@
 2. Within each group rows are sorted by score descending; ties break by recency.
 3. When the top result across all groups scores &gt; 0.95 (an ID match) it is pinned as a single row above the groups, carrying its entity icon.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), the section/story named in this case's References, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), the section/story named in this case's References, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2038,7 +2038,7 @@
 4. A date is shown (for example 'Apr 27, 2026').
 5. A briefcase / work-order icon is shown on the left of the row.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 4 Work Orders (Displayed: WO number + customer, status badge, lead technician, asset/unit, date), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 4 Work Orders (Displayed: WO number + customer, status badge, lead technician, asset/unit, date), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2090,7 +2090,7 @@
 3. A count chip is shown (the open work-order / document count, for example '12').
 4. A person icon is shown on the left of the row.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 4 Customers (Displayed: name, address line, open WO count badge, telephone on hover), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 4 Customers (Displayed: name, address line, open WO count badge, telephone on hover), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2141,7 +2141,7 @@
 2. The owning customer name is shown as smaller secondary text (for example 'Bryan Smith').
 3. A vehicle icon is shown on the left of the row.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 4 Assets (Displayed: year + make + model primary, customer name secondary), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 4 Assets (Displayed: year + make + model primary, customer name secondary), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2194,7 +2194,7 @@
 4. The quantity chip is colored by stock status: green when in stock, orange when low, red when out of stock.
 5. A tag / part icon is shown on the left of the row.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 4 Parts (Displayed: description, part number, total quantity with stock-status color), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 4 Parts (Displayed: description, part number, total quantity with stock-status color), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2245,7 +2245,7 @@
 2. An address line is shown as the secondary line.
 3. A building icon is shown on the left of the row.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 4 Vendors (Displayed: vendor name primary, address line secondary), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 4 Vendors (Displayed: vendor name primary, address line secondary), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2297,7 +2297,7 @@
 3. A total price and a created date are shown.
 4. A label icon is shown on the left of the row.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 4 Part Sales (Displayed: P-number + customer primary, status badge, total price + created date), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 4 Part Sales (Displayed: P-number + customer primary, status badge, total price + created date), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2348,7 +2348,7 @@
 2. Its secondary line shows 'Contact match' to indicate the match was on a contact field (phone or email) rather than the name.
 3. When the query reaches both a contact and its parent company, two rows are returned - the contact in the Contacts group and the company in its own group carrying the 'Contact match' label; neither row suppresses the other.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 4 (contact-field match), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 4 (contact-field match), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2398,7 +2398,7 @@
           <t>1. Status badge colors match the Work Order list tokens: Approved green, Estimate blue, Review yellow, In Progress blue, Completed gray, Declined red, Invoiced purple.
 2. Part stock badges use green (available), orange (low), red (out).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.3 (status badge colors, same tokens as the WO list), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.3 (status badge colors, same tokens as the WO list), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2448,7 +2448,7 @@
           <t>1. The 'Peterson' record is found and shown, despite the typo.
 2. The matched part of the text is highlighted.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 7 (token n-gram / trigram matching catches Petersn -&gt; Peterson), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 7 (token n-gram / trigram matching catches Petersn -&gt; Peterson), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2497,7 +2497,7 @@
         <is>
           <t>1. The 'Aabridge' record is found and shown, despite the typo.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 1 + 10 Phase 5 (fuzzy query 'Abrige'), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 1 + 10 Phase 5 (fuzzy query 'Abrige'), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2546,7 +2546,7 @@
         <is>
           <t>1. The 'Freightliner' record is found and shown, despite the transposed letters.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 7 (Damerau-Levenshtein; freihgtliner -&gt; freightliner), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 7 (Damerau-Levenshtein; freihgtliner -&gt; freightliner), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2595,7 +2595,7 @@
         <is>
           <t>1. The 'Fibridge' record is found and shown (matched by sound, as a last-resort phonetic match), likely lower in the ranking than an exact/near-exact match.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 7 (phonetic fallback catches Filbridge -&gt; Fibridge), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 7 (phonetic fallback catches Filbridge -&gt; Fibridge), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2647,7 +2647,7 @@
 2. The Work Order number is treated as an identifier: it is normalized by stripping the dash/space, so 'S2-15276' equals 's215276'.
 3. The match is exact (identifier), not fuzzy.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 7 (S2-15276 = s215276); identifier fields are exact-only, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 7 (S2-15276 = s215276); identifier fields are exact-only, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2697,7 +2697,7 @@
           <t>1. The exact VIN (case and spacing normalized) finds the matching asset / work order.
 2. A VIN with a wrong character does NOT return a fuzzy match - VINs are exact-only identifiers, no typo tolerance.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 7 (What is NOT fuzzy: VIN, WO number, P-number, part number - exact match after normalization), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 7 (What is NOT fuzzy: VIN, WO number, P-number, part number - exact match after normalization), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2748,7 +2748,7 @@
 2. The phone is normalized to digits only, so '(264) 328-6723' equals '2643286723'.
 3. The matched customer's secondary line shows 'Contact/info match' (matched on a contact field, not the name).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 7 (phone normalization); 4 (Contact/info match affordance), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 7 (phone normalization); 4 (Contact/info match affordance), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2798,7 +2798,7 @@
           <t>1. The exact part number finds the matching part.
 2. A part number with a wrong digit does NOT return a fuzzy match - part numbers are exact-only identifiers.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 7 (What is NOT fuzzy: part number), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 7 (What is NOT fuzzy: part number), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2848,7 +2848,7 @@
           <t>1. The real Work Order 'S2-15276' is NOT returned as a fuzzy match.
 2. Because identifier fields are exact-only, a one-digit-off WO number returns no fuzzy identifier match (it may show 'No results' if nothing else matches).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 7 (exact identifier fields bypass fuzzy logic), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 7 (exact identifier fields bypass fuzzy logic), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2898,7 +2898,7 @@
           <t>1. The matched token is highlighted.
 2. A subtle soft-match indicator is shown for fuzzy matches (spec mentions a '≈' symbol or italic treatment).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 7 (fuzzy soft-match highlight treatment - design polish, confirm with design), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 7 (fuzzy soft-match highlight treatment - design polish, confirm with design), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2948,7 +2948,7 @@
           <t>1. The exact P-number 'P2-58' finds the matching Part Sale.
 2. A one-digit-off P-number does NOT return the real Part Sale as a fuzzy match - P-numbers are exact-only identifiers, no typo tolerance (it may show 'No results' if nothing else matches).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 7 (What is NOT fuzzy: VIN, WO number, P-number, part number - exact match after normalization), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 7 (What is NOT fuzzy: VIN, WO number, P-number, part number - exact match after normalization), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -2998,7 +2998,7 @@
           <t>1. The exactly-matched Work Order is pinned as a single row at the very top, above the grouped results, labeled with its entity icon.
 2. This gives the 'type the number, jump straight to it' experience.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 6.2 (ID match &gt; 0.95 pinned at top), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 6.2 (ID match &gt; 0.95 pinned at top), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3048,7 +3048,7 @@
           <t>1. Open/active and recently-updated Work Orders rank above old, closed ones.
 2. Work Orders assigned to or recently viewed by the signed-in user are boosted; closed/Invoiced Work Orders older than 90 days are pushed down.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 6.1 Work Orders signals (open status +0.30, recency, assigned/viewed, old-closed demoted), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 6.1 Work Orders signals (open status +0.30, recency, assigned/viewed, old-closed demoted), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3098,7 +3098,7 @@
           <t>1. The in-stock part ranks above the out-of-stock part.
 2. The out-of-stock part is still shown (out-of-stock parts are not demoted below relevance and are not hidden).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 6.1 Parts signals, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 6.1 Parts signals, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3148,7 +3148,7 @@
           <t>1. Assets and Work Orders owned by the customer whose page you are on are boosted (appear higher) compared to the same search run from an unrelated page.
 2. This is a lightweight, single contextual-bias signal.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 6.3 Contextual bias, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 6.3 Contextual bias, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3198,7 +3198,7 @@
           <t>1. Parts already on that work order are pushed down (demoted) relative to other matching parts.
 2. Other parts in the same category as the work order's existing parts get a small boost.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 6.3 Contextual bias, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 6.3 Contextual bias, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3247,7 +3247,7 @@
 2. More recently created POs rank above older ones (recency decays over about two weeks).
 3. A PO created by the signed-in user gets a small additional boost.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), 6.1 (Purchase Order signals), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), 6.1 (Purchase Order signals), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3295,7 +3295,7 @@
           <t>1. An Unpaid vendor invoice ranks above paid ones.
 2. More recent invoice dates rank higher (recency decays over about a month).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), 6.1 (Vendor Invoice signals), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), 6.1 (Vendor Invoice signals), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3344,7 +3344,7 @@
 2. A contact called or viewed by the signed-in user in the last 7 days gets a boost.
 3. A company's primary contact gets a small additional boost.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), 6.1 (Contact signals), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), 6.1 (Contact signals), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3396,7 +3396,7 @@
 3. Three quick-create buttons are shown: 'New work order', 'New customer', 'New inventory part'.
 4. The footer keyboard legend is visible: down/up Navigate, Enter Select, Esc Close.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.1 / 5.2 (first-time state and placeholder copy), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.1 / 5.2 (first-time state and placeholder copy), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3448,7 +3448,7 @@
 3. 'New inventory part' starts the create-inventory-part flow.
 4. None of the buttons perform a destructive action.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 State 1 (quick-create chips), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 State 1 (quick-create chips), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3499,7 +3499,7 @@
 2. Rows are grouped under time headings: 'Today', 'Yesterday', 'Past week', 'Past 30 days'.
 3. Each row is a previously opened record (not just a previous search word).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 State 2 (Recent searches grouped by interval); 8 (persist recent-entity-views 30 days), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 State 2 (Recent searches grouped by interval); 8 (persist recent-entity-views 30 days), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3550,7 +3550,7 @@
 2. Each recent row uses the same row template as a normal result row (icon, primary line, secondary line, status/quantity cluster).
 3. Example rows: WO 'S1-644 Fisquare Farms' [Approved], Asset '2025 Freightliner M2 - Bryan Smith', Customer 'Adale Transport' with a doc chip, Part 'Rear Shock 65547' [72], Vendor 'Report Beverages'.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 State 2 (same row template as a result row), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 State 2 (same row template as a result row), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3599,7 +3599,7 @@
           <t>1. The palette closes and the clicked record opens.
 2. Opening the record refreshes its position in recent activity (it is 'touched').
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 10 Phase 4 (records a touch on every result click / entity-page visit), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 10 Phase 4 (records a touch on every result click / entity-page visit), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3649,7 +3649,7 @@
 3. After clearing, the panel falls back to the first-time state - helper text plus the three quick-create buttons - with no separate empty-history message.
 4. 'Clear all' is present on both web and mobile.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), 5.2 / 5.6 / 8 (Clear all), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), 5.2 / 5.6 / 8 (Clear all), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3702,7 +3702,7 @@
 3. The list is deduplicated: re-viewing an entity moves it to the top rather than adding a duplicate.
 4. A deleted entity is excluded from the recents list.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), the section/story named in this case's References, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), the section/story named in this case's References, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3753,7 +3753,7 @@
           <t>1. After closing, the header search field still shows the last query 'Fibridge' as plain text.
 2. A small count badge (for example '1') is shown beside the persisted query.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 State 5 (Persisting search); 8 (persist last query, rehydrate on reopen), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 State 5 (Persisting search); 8 (persist last query, rehydrate on reopen), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3804,7 +3804,7 @@
 3. The result list for that query is shown again.
 4. The query text may appear selected/highlighted in the input so it can be replaced by typing.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 State 5 (Reopening restores the query, the scope tab, and the result list), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 State 5 (Reopening restores the query, the scope tab, and the result list), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3854,7 +3854,7 @@
 2. The results clear and the palette returns to the empty / recent-activity state (placeholder a plain search placeholder (no 'ask a question' / AI wording in v1 - exact copy per the v2 design)).
 3. The persisted query is removed from the header field.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 State 5; design-notes screenshot 9 (clearable via the x button), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 State 5; design-notes screenshot 9 (clearable via the x button), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3905,7 +3905,7 @@
 2. The three quick-create buttons are shown: 'New work order', 'New customer', 'New inventory part'.
 3. The footer keyboard legend is still visible.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 State 4 (No results for [query] + quick-create chips), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 State 4 (No results for [query] + quick-create chips), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -3954,7 +3954,7 @@
           <t>1. The matching create flow starts (create work order / customer / inventory part).
 2. No destructive action occurs.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.2 State 4, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.2 State 4, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4006,7 +4006,7 @@
 3. A 'Clear search' link appears on the right of the banner.
 4. The list columns remain: On Site, Status, Number, Customer, Asset, Unit, VIN/Serial #, Progress, Service Advisor, Lead Technician, Clocked In, Lines, Total Price.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), design-notes screenshot 1 (in-page Work Orders list search banner), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), design-notes screenshot 1 (in-page Work Orders list search banner), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4055,7 +4055,7 @@
           <t>1. The filter is removed and the full Work Orders list is shown again.
 2. The 'Showing N work orders matching [q]' banner is removed.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), design-notes screenshot 1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), design-notes screenshot 1, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4107,7 +4107,7 @@
 2. The palette degrades gracefully - it does not crash or show a blank screen.
 3. Retrying after connectivity is restored re-runs the search and shows results.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 8 (tolerate offline/network failures with an inline 'Search unavailable, retry' banner), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 8 (tolerate offline/network failures with an inline 'Search unavailable, retry' banner), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4157,7 +4157,7 @@
           <t>1. A 'Parts' group appears with matching part rows.
 2. The 'Parts' scope tab shows the part results.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 9 (all result fields respect role-based-access checks), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 9 (all result fields respect role-based-access checks), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4208,7 +4208,7 @@
 2. The user cannot see part results they are not permitted to access, even though those parts exist.
 3. Results for entity types the user CAN access still appear normally.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 9 (a technician without Parts access does not see Parts results), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 9 (a technician without Parts access does not see Parts results), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4258,7 +4258,7 @@
           <t>1. No 'Work orders' group appears and no Work Order rows are shown.
 2. Results for entity types the user CAN access still appear normally.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 9 (all result fields respect role-based-access checks), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 9 (all result fields respect role-based-access checks), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4308,7 +4308,7 @@
           <t>1. Only records belonging to your own tenant/organization are returned.
 2. No records from any other tenant are shown (tenant isolation is respected).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 9 (all result fields respect existing tenant-isolation checks), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 9 (all result fields respect existing tenant-isolation checks), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4360,7 +4360,7 @@
 2. Groups for the entity types that do have matches still appear normally.
 3. The empty entity type's scope tab shows its empty / no-results treatment rather than an error.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 9 (must work for a single-tenant dataset where any entity type is empty, e.g. no part sales yet), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 9 (must work for a single-tenant dataset where any entity type is empty, e.g. no part sales yet), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4413,7 +4413,7 @@
 3. Without See Financial Data every price field is masked in results (part purchase/sell price, part-sale total, WO total, PO total, vendor-invoice total); masked values are never sent in the response.
 4. The TimeClock role gets an empty result set.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), the section/story named in this case's References, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), the section/story named in this case's References, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4464,7 +4464,7 @@
 2. The body is a grouped, ranked, scored payload containing groups for the matching entity types.
 3. Each group includes the per-item metadata needed to render rows without extra fetches.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 10 Phase 1 (GET /api/search; scope=all), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 10 Phase 1 (GET /api/search; scope=all), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4516,7 +4516,7 @@
 2. Each response contains results only for the requested scope's entity type.
 3. The accepted scope values are all, work_orders, customers, assets, parts, vendors, part_sales.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 10 Phase 1 (scope parameter), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 10 Phase 1 (scope parameter), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4568,7 +4568,7 @@
 2. Each group reports its full total count (for example total 12) even though only 5 rows are returned.
 3. Setting limit changes the per-group cap accordingly.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 10 Phase 1 (limit default 5; response includes per-group totals), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 10 Phase 1 (limit default 5; response includes per-group totals), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4621,7 +4621,7 @@
 2. The identifier is normalized (case, diacritics, non-alphanumerics stripped) before matching.
 3. The exact-match result scores high enough to be flagged as the pinned top match (score above 0.95).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 7 (identifier normalization); 6.2 (ID match pinned), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 7 (identifier normalization); 6.2 (ID match pinned), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4671,7 +4671,7 @@
           <t>1. The real Work Order 'S2-15276' is NOT returned as a fuzzy identifier match.
 2. Identifier fields (VIN, WO number, P-number, part number) require exact match after normalization; fuzzy logic is bypassed for them.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 7 (What is NOT fuzzy), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 7 (What is NOT fuzzy), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4723,7 +4723,7 @@
 2. Scoping directly to 'parts' still returns no forbidden parts (empty or a permission-appropriate response).
 3. Entity types the user is allowed to access are still returned.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 9 (results respect role-based-access checks - enforced server-side), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 9 (results respect role-based-access checks - enforced server-side), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4775,7 +4775,7 @@
 2. A backend failure returns a 5xx or error payload that the frontend maps to the inline 'Search unavailable, retry' banner.
 3. The endpoint fails gracefully rather than returning malformed data.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 8 (offline/network failure handling), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 8 (offline/network failure handling), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4826,7 +4826,7 @@
 2. Within each group items are ordered by score descending; ties break by recency.
 3. Each item carries the metadata needed to render its row (entity type, primary/secondary fields, badges/quantity, score) without extra fetches, and true per-group totals.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 6.2 (group order); 10 Phase 1 (per-item metadata), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 6.2 (group order); 10 Phase 1 (per-item metadata), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4878,7 +4878,7 @@
 2. Passing the cursor returns the next page of scoped results (no duplicates, no gaps).
 3. Pagination applies to the scoped-tab view.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 10 Phase 1 (cursor parameter), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 10 Phase 1 (cursor parameter), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4929,7 +4929,7 @@
           <t>1. With the customer context, assets and work orders owned by that customer are boosted in the ranking versus the no-context call.
 2. The context parameter takes an optional {type, id} for page-context bias.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 6.3 (contextual bias); 10 Phase 1 (context parameter), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 6.3 (contextual bias); 10 Phase 1 (context parameter), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -4980,7 +4980,7 @@
 2. GET /user/recent-entities returns the recently touched records, retained for 30 days.
 3. The results support bucketing into Today / Yesterday / Past week / Past 30 days at render time.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 8 (persist recent-entity-views 30 days); 10 Phase 4, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 8 (persist recent-entity-views 30 days); 10 Phase 4, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5031,7 +5031,7 @@
           <t>1. The backend is not queried on every keystroke; input is debounced (about 150ms) so a request fires after a short pause.
 2. Grouped results render quickly once the response arrives (target within about 200ms at p95).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 8 (debounce input at 150ms; render within 200ms p95), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 8 (debounce input at 150ms; render within 200ms p95), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5083,7 +5083,7 @@
 3. A contact row carries the contact (user-round) icon, the contact name (primary), and its company/context (secondary); a match on phone/email carries the "Contact/info match" flag.
 4. Company-less contacts (no company_id) are not indexed and do not appear.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), the section/story named in this case's References, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), the section/story named in this case's References, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5135,7 +5135,7 @@
 3. Adding a new searchable entity is a single provider class plus mapping (framework extensibility), so page and global search stay in lockstep.
 4. Exports keep their current data path in v1 (not cut over).
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), the section/story named in this case's References, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), the section/story named in this case's References, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5186,7 +5186,7 @@
 2. The old GET /api/global-search/fetch endpoint, its handler and the client-side filtering are removed after stabilisation.
 3. The 3-result-per-category dropdown behaviour is replaced entirely by the modal.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), the section/story named in this case's References, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), the section/story named in this case's References, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5237,7 +5237,7 @@
 2. The action is non-destructive.
 ---
 EXCLUDED FROM V1 - not tested in this release. Contextual quick actions on result rows are a v1 non-goal: the Global Search PRD v1.2 documents the intended behaviour in section 5.4 but states it “is not part of the v1 build and carries no v1 stories” (see also section 2, Non-Goals). Kept for the future release in which quick actions are built - do not execute against the v1 build.
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.4 (Work Order -&gt; 'Add new line', only when currently editing a WO elsewhere), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.4 (Work Order -&gt; 'Add new line', only when currently editing a WO elsewhere), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5289,7 +5289,7 @@
 3. The actions are non-destructive.
 ---
 EXCLUDED FROM V1 - not tested in this release. Contextual quick actions on result rows are a v1 non-goal: the Global Search PRD v1.2 documents the intended behaviour in section 5.4 but states it “is not part of the v1 build and carries no v1 stories” (see also section 2, Non-Goals). Kept for the future release in which quick actions are built - do not execute against the v1 build.
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.4 (Asset -&gt; 'New work order' + clock (history) and Invoice icons), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.4 (Asset -&gt; 'New work order' + clock (history) and Invoice icons), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5341,7 +5341,7 @@
 3. The actions are non-destructive.
 ---
 EXCLUDED FROM V1 - not tested in this release. Contextual quick actions on result rows are a v1 non-goal: the Global Search PRD v1.2 documents the intended behaviour in section 5.4 but states it “is not part of the v1 build and carries no v1 stories” (see also section 2, Non-Goals). Kept for the future release in which quick actions are built - do not execute against the v1 build.
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.4 (Customer -&gt; 'New work order', 'New contact'), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.4 (Customer -&gt; 'New work order', 'New contact'), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5394,7 +5394,7 @@
 3. The action is non-destructive.
 ---
 EXCLUDED FROM V1 - not tested in this release. Contextual quick actions on result rows are a v1 non-goal: the Global Search PRD v1.2 documents the intended behaviour in section 5.4 but states it “is not part of the v1 build and carries no v1 stories” (see also section 2, Non-Goals). Kept for the future release in which quick actions are built - do not execute against the v1 build.
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.4 (Part -&gt; 'Add part' when not currently editing a WO), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.4 (Part -&gt; 'Add part' when not currently editing a WO), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5445,7 +5445,7 @@
 2. The action is non-destructive.
 ---
 EXCLUDED FROM V1 - not tested in this release. Contextual quick actions on result rows are a v1 non-goal: the Global Search PRD v1.2 documents the intended behaviour in section 5.4 but states it “is not part of the v1 build and carries no v1 stories” (see also section 2, Non-Goals). Kept for the future release in which quick actions are built - do not execute against the v1 build.
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.4 (Vendor -&gt; 'Add contact'), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.4 (Vendor -&gt; 'Add contact'), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5497,7 +5497,7 @@
 2. Using it adds the part to the work order you are editing (an inline add, non-destructive).
 ---
 EXCLUDED FROM V1 - not tested in this release. Contextual quick actions on result rows are a v1 non-goal: the Global Search PRD v1.2 documents the intended behaviour in section 5.4 but states it “is not part of the v1 build and carries no v1 stories” (see also section 2, Non-Goals). Kept for the future release in which quick actions are built - do not execute against the v1 build.
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.4 (Part -&gt; 'Add to work order' only when currently editing a WO), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.4 (Part -&gt; 'Add to work order' only when currently editing a WO), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5547,7 +5547,7 @@
 2. Every action offered by a quick action is also reachable from the entity's full record (hover is non-essential).
 ---
 EXCLUDED FROM V1 - not tested in this release. Contextual quick actions on result rows are a v1 non-goal: the Global Search PRD v1.2 documents the intended behaviour in section 5.4 but states it “is not part of the v1 build and carries no v1 stories” (see also section 2, Non-Goals). Kept for the future release in which quick actions are built - do not execute against the v1 build.
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.4 (Quick actions never trigger destructive operations; hover state non-essential), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.4 (Quick actions never trigger destructive operations; hover state non-essential), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5599,7 +5599,7 @@
 3. The "currently editing a WO" state comes from the shared page-context source.
 ---
 EXCLUDED FROM V1 - not tested in this release. Contextual quick actions on result rows are a v1 non-goal: the Global Search PRD v1.2 documents the intended behaviour in section 5.4 but states it “is not part of the v1 build and carries no v1 stories” (see also section 2, Non-Goals). Kept for the future release in which quick actions are built - do not execute against the v1 build.
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), the section/story named in this case's References, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), the section/story named in this case's References, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5652,7 +5652,7 @@
 3. Quick actions remain reachable on touch (no hover) via the design's touch affordance.
 4. The tab strip remains usable with up to ten tabs on a narrow viewport.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), the section/story named in this case's References, read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), the section/story named in this case's References, read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5702,7 +5702,7 @@
 3. The placeholder copy is 'Search everything'.
 4. There is no keyboard-hints footer on mobile.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), 5.6 (mobile surface), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), 5.6 (mobile surface), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5751,7 +5751,7 @@
 2. The chip row appears only once there is a query.
 3. It lists only the entity types that actually matched, each with its count, so the row stays short.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), 5.6 (mobile scope chips), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), 5.6 (mobile scope chips), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5801,7 +5801,7 @@
 3. Group headers stick to the top of the list while scrolling.
 4. A tap on a row opens the record.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), 5.6 (mobile results), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), 5.6 (mobile results), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5850,7 +5850,7 @@
 2. The quick-create buttons are stacked full-width instead of inline.
 3. 'Clear all' behaves as on web: clearing the history returns the screen to the first-time state.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), 5.6 (mobile states), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), 5.6 (mobile states), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5898,7 +5898,7 @@
           <t>1. The full-page result handoff and its banner (the web 'Show all' behaviour) do not apply on mobile in v1 - the mobile lists have no query handoff.
 2. Keyboard navigation does not apply on mobile.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), 5.6 (mobile deferrals), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), 5.6 (mobile deferrals), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -5949,7 +5949,7 @@
 2. A PO row carries the package icon; the primary line shows the PO number + vendor, and the row shows a status badge (Ordered / Received) with the total and created date.
 3. PO results are gated by Vendor &amp; Order Management: View.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.3 / 6.1 (Purchase Orders row), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.3 / 6.1 (Purchase Orders row), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -6001,7 +6001,7 @@
 3. This is mechanism/schema only - no ML ranking model is expected in v1.
 4. SCOPE NOTE (PO-GS-5): the owning story SV-9167 is currently in the backlog. If event logging is not present on the build, record it as a deviation to raise with Product - do not silently pass or ignore it.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 8 (functional requirements) / 6.4 (telemetry schema), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 8 (functional requirements) / 6.4 (telemetry schema), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>
@@ -6053,7 +6053,7 @@
 3. The payment status badge per the spec (section 5.3) is Paid or Unpaid. KNOWN VARIANCE (PO-GS-6): if the build shows a third 'Partially paid' state, treat it as an expected variance to confirm with Product - do NOT fail the case on it.
 4. Vendor Invoice results are gated by Vendor &amp; Order Management: View, and the invoice total is masked for a user without See Financial Data.
 ---
-This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 11), section 5.3 / 6.1 (Vendor Invoices row), read on 25 August 2026.
+This is the expected behaviour as per epic SV-9160 and the Global Search - Product Requirements specification version 1.2 (Confluence page 576978945, Confluence version 12), section 5.3 / 6.1 (Vendor Invoices row), read on 26 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/25/2026</t>
         </is>
       </c>

</xml_diff>